<commit_message>
Renewal FRS, comparison and coverage workbooks regenerated: every FR item and acceptance criterion available, notices added to Annex AE, configurable points marked for BDOI to confirm the setting
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>9 October 2026</t>
+          <t>10 October 2026</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Keep Clean / Review / Exception as the BRD says; show the Not for Renewal accounts as BDOI's "Non-Renewable" panel (a filter on the disposition). (BIBS reference FRS: FR-RN-022: buckets Clean, Review and Exception; missing mandatory data is a sanitation failure (Exception). The system today: Clean, Review, Exception.)</t>
+          <t>Keep Clean / Review / Exception as the BRD says; show the Not for Renewal accounts as BDOI's "Non-Renewable" panel (a filter on the disposition). (BIBS reference FRS: FR-RN-022: buckets Clean, Review and Exception; missing mandatory data is a sanitation failure (Exception). The system today: Clean, Review, Exception.) Available in BIBS: the third panel of the renewal accounts is Non-Renewable (default, BDOI's panels Clean, Review, Non-Renewable and All, the Exception accounts shown under Review) or Exception (the BRD's Clean, Review and Exception).</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Keep the Review bucket (the TSU route is manual work) and use BDOI's disposition word once the For Quotation / For Proposal meaning is settled. (BIBS reference FRS: FR-RN-020: above PHP 250M the renewal account is Review and the decision matrix proposes For Proposal to TSU. The system today: Review with a proposed disposition.)</t>
+          <t>Keep the Review bucket (the TSU route is manual work) and use BDOI's disposition word once the For Quotation / For Proposal meaning is settled. (BIBS reference FRS: FR-RN-020: above PHP 250M the renewal account is Review and the decision matrix proposes For Proposal to TSU. The system today: Review with a proposed disposition.) Available in BIBS: an account above the sum insured threshold is Clean For Quotation and goes to the TSU (default, BDOI's rule) or Review with a proposal for the TSU.</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Keep the Team Lead assignment of the BRD and add automatic assignment as an option per segment (change to the system), if BDOI confirms. (BIBS reference FRS: FR-RN-030, 061: the Team Lead assigns and re-assigns; CBG accounts are not assigned. The system today: Manual assignment.)</t>
+          <t>Keep the Team Lead assignment of the BRD and add automatic assignment as an option per segment (change to the system), if BDOI confirms. (BIBS reference FRS: FR-RN-030, 061: the Team Lead assigns and re-assigns; CBG accounts are not assigned. The system today: Manual assignment.) Available in BIBS: the renewal accounts of the market segments chosen are assigned automatically to an Account Officer of the team, fewest open accounts first and then in turn, and the accounts routed to Processing to a Processing Officer when a second setting is on; with no segment chosen (default, the BRD) the Team Leader assigns.</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD transfer; add BDOI's referral as a second action (New Business opportunity) if BDOI wants both. (BIBS reference FRS: FR-RN-031, 032: the renewal moves to the receiving unit when it accepts. The system today: Ownership transfer.)</t>
+          <t>Keep the BRD transfer; add BDOI's referral as a second action (New Business opportunity) if BDOI wants both. (BIBS reference FRS: FR-RN-031, 032: the renewal moves to the receiving unit when it accepts. The system today: Ownership transfer.) Available in BIBS: a transfer to another Marketing unit is a referral (the receiving unit opens a New Business account and the renewal keeps its owner, BDOI's text), a move of the account (the BRD), or both offered to the user (default).</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Keep the RA lock of the BRD and add BDOI's lock after placement (edits after placement are already refused by the account). (BIBS reference FRS: FR-RN-080: RA generation locks the account on the Marketing side; an RA cancellation unlocks it. The system today: Lock at RA generation.)</t>
+          <t>Keep the RA lock of the BRD and add BDOI's lock after placement (edits after placement are already refused by the account). (BIBS reference FRS: FR-RN-080: RA generation locks the account on the Marketing side; an RA cancellation unlocks it. The system today: Lock at RA generation.) Available in BIBS: Marketing can no longer change the account once the Renewal Advice is generated (default, BDOI's text) or once it is posted and the placement is sent.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's durations as parameters now; automatic requests and extensions are a change to the system for BDOI to prioritise. (BIBS reference FRS: FR-RN-086: the user requests 30 or 60 days (default 30) when the renewal will not complete in time. The system today: User request, 30 or 60 days.)</t>
+          <t>Adopt BDOI's durations as parameters now; automatic requests and extensions are a change to the system for BDOI to prioritise. (BIBS reference FRS: FR-RN-086: the user requests 30 or 60 days (default 30) when the renewal will not complete in time. The system today: User request, 30 or 60 days.) Available in BIBS: hold cover durations of 30 days (Non-CBG), 90 days (CBG), 60 days (CBG Motor after an insurer's rejection) and 30 days (CBG Home), extensions of 15 or 30 days from 7 days before the end, automatic requests for Non-CBG accounts after the client's confirmation and for Clean CBG accounts 75 days before expiry, and the monthly CBG Home extension on the 15th; each value is a setting.</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's 75 / 45 days and the automatic determination; name the notices First and Final as in the approved templates. (BIBS reference FRS: FR-RN-080: the user chooses First or Second Notice; second notice after 15 days without acceptance; warning below 30 days. The system today: User choice; second-notice days parameter.)</t>
+          <t>Adopt BDOI's 75 / 45 days and the automatic determination; name the notices First and Final as in the approved templates. (BIBS reference FRS: FR-RN-080: the user chooses First or Second Notice; second notice after 15 days without acceptance; warning below 30 days. The system today: User choice; second-notice days parameter.) Available in BIBS: the Renewal Advice notice follows the expiry, First Notice from 75 days and Last Notice from 45 days before expiry (default, BDOI's text), or is chosen by the user.</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Keep the mutual exclusion and the effective expiry date of the BRD; adopt BDOI's day offsets (1 and 3 days) as parameters. (BIBS reference FRS: FR-RN-082: at the effective expiry date (hold cover end), NAL when an RA was sent, NRL when none; the two exclude each other. The system today: Mutually exclusive, effective expiry date.)</t>
+          <t>Keep the mutual exclusion and the effective expiry date of the BRD; adopt BDOI's day offsets (1 and 3 days) as parameters. (BIBS reference FRS: FR-RN-082: at the effective expiry date (hold cover end), NAL when an RA was sent, NRL when none; the two exclude each other. The system today: Mutually exclusive, effective expiry date.) Available in BIBS: the No Advice Letter 1 day and the Non-Renewal Letter 1 day (CBG Motor) or 3 days (Non-CBG) after the effective expiry date, each a setting; the two letters exclude each other.</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's convention (answers Q07); change to the system of the password rule. (BIBS reference FRS: FR-RN-081: password convention per Q07; until then a generated password per e-mail. The system today: Random 12-character password in a separate e-mail.)</t>
+          <t>Adopt BDOI's convention (answers Q07); change to the system of the password rule. (BIBS reference FRS: FR-RN-081: password convention per Q07; until then a generated password per e-mail. The system today: Random 12-character password in a separate e-mail.) Available in BIBS: protected files use BDOI's password convention (default: the first three letters of the first and last names in capitals for an individual client, eight random characters for a corporate client) or a random password per file.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>BDO ITG decides whether CCM and MFT are in scope for go-live; the system keeps e-mail as the fallback channel. (BIBS reference FRS: Outgoing e-mail, protected, with a send log; no file-transfer channel with insurers (on hold). The system today: Outgoing e-mail; CCM listed as an option in the integration inventory (IQ11).)</t>
+          <t>BDO ITG decides whether CCM and MFT are in scope for go-live; the system keeps e-mail as the fallback channel. (BIBS reference FRS: Outgoing e-mail, protected, with a send log; no file-transfer channel with insurers (on hold). The system today: Outgoing e-mail; CCM listed as an option in the integration inventory (IQ11).) Available in BIBS: client documents are sent through CCM (default) or by protected e-mail with the password in a separate e-mail; insurers receive their files through MFT when enrolled, otherwise by e-mail.</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Keep the booking a user action as the Walkthrough addendum says, unless BDOI changes it. (BIBS reference FRS: FR-RN-084: placement and booking stay user actions. The system today: Booking is a user action (automatic booking rules exist in New Business).)</t>
+          <t>Keep the booking a user action as the Walkthrough addendum says, unless BDOI changes it. (BIBS reference FRS: FR-RN-084: placement and booking stay user actions. The system today: Booking is a user action (automatic booking rules exist in New Business).) Available in BIBS: the insurer's approval of the placement leaves the account For Booking for the Processing Officer (default, the BRD) or books and locks it (BDOI's text).</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Keep ours and add BDOI's Review routing for endorsements of the term if Marketing wants to see them. (BIBS reference FRS: FR-RN-027: posted endorsements are taken into the renewal; an endorsement in progress blocks post, RA and acceptance. The system today: Pending endorsement blocks.)</t>
+          <t>Keep ours and add BDOI's Review routing for endorsements of the term if Marketing wants to see them. (BIBS reference FRS: FR-RN-027: posted endorsements are taken into the renewal; an endorsement in progress blocks post, RA and acceptance. The system today: Pending endorsement blocks.) Available in BIBS: every endorsement of the expiring term routes the account to Review (default, BDOI's text) or only an endorsement in progress.</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Keep the five dispositions of the BRD and add BDOI's eleven extra reasons as list values. (BIBS reference FRS: FR-RN-043: five dispositions (with Lost Business) and ten reasons. The system today: Five dispositions; eleven reasons (list values).)</t>
+          <t>Keep the five dispositions of the BRD and add BDOI's eleven extra reasons as list values. (BIBS reference FRS: FR-RN-043: five dispositions (with Lost Business) and ten reasons. The system today: Five dispositions; eleven reasons (list values).) Available in BIBS: the dispositions offered to Marketing are For Renewal, Not for Renewal, For Quotation, For Proposal and Lost Business (default, the BRD) or the first four with Lost Business as a reason of Not for Renewal (BDOI's text); BDOI's non-renewal reasons are in the list of values.</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Ask BDOI; a second approval is a change to the system and slows BRRN.040. (BIBS reference FRS: FR-RN-084: the accepted account moves to placement and booking without resubmission. The system today: No second approval.)</t>
+          <t>Ask BDOI; a second approval is a change to the system and slows BRRN.040. (BIBS reference FRS: FR-RN-084: the accepted account moves to placement and booking without resubmission. The system today: No second approval.) Available in BIBS: an accepted account goes to the payment check and placement at once (default, the BRD) or is Submitted for Approval and goes to placement once an approver approves it (BDOI's text).</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Keep the matrix and load BDOI's rule (Clean is automatic For Renewal) as its first content. (BIBS reference FRS: FR-RN-023: the decision matrix gives a system disposition to Clean accounts whose rule is automatic; others are proposed to the AO; the Team Lead posts. The system today: Matrix proposal or automatic disposition.)</t>
+          <t>Keep the matrix and load BDOI's rule (Clean is automatic For Renewal) as its first content. (BIBS reference FRS: FR-RN-023: the decision matrix gives a system disposition to Clean accounts whose rule is automatic; others are proposed to the AO; the Team Lead posts. The system today: Matrix proposal or automatic disposition.) Available in BIBS: Clean accounts are disposed For Renewal automatically (default, BDOI's rule) or wait for the disposition of Marketing.</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Map the two lists one to one in the status model annex and use BDOI's names where the BRD is silent. (BIBS reference FRS: Extracted, Evaluating, Unassigned Disposition, For Disposition, Review in Progress, For Processing, With Insurer, RA Ready, RA Sent, Accepted, For Placement and Booking, Renewed, Closed. The system today: The the system stages.)</t>
+          <t>Map the two lists one to one in the status model annex and use BDOI's names where the BRD is silent. (BIBS reference FRS: Extracted, Evaluating, Unassigned Disposition, For Disposition, Review in Progress, For Processing, With Insurer, RA Ready, RA Sent, Accepted, For Placement and Booking, Renewed, Closed. The system today: The the system stages.) Available in BIBS: the statuses read with BDOI's names (default: In Process Renewal, Submitted for Posting, Posted and the others) or with the workflow status names.</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Use BDOI's names RMEL and NRL in the merged FRS and on the screens. (BIBS reference FRS: Expiry List; Not for Renewal Letter (NFR). The system today: Expiry List; NAL / NFR.)</t>
+          <t>Use BDOI's names RMEL and NRL in the merged FRS and on the screens. (BIBS reference FRS: Expiry List; Not for Renewal Letter (NFR). The system today: Expiry List; NAL / NFR.) Available in BIBS: generated files are named with BDOI's convention &lt;Product&gt;_&lt;Letter&gt;_&lt;Reference&gt;_MMDDYYYY.pdf (default) or with the letter number.</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD label and correct BDOI's two variants. (BIBS reference FRS: FR-RN-024: "Non-renewable Accounts". The system today: Non-renewable Accounts.)</t>
+          <t>Keep the BRD label and correct BDOI's two variants. (BIBS reference FRS: FR-RN-024: "Non-renewable Accounts". The system today: Non-renewable Accounts.) Available in BIBS: the reason recorded for a non-renewable risk code is Non-renewable Accounts (default, the BRD) or Non-Renewable Risk Code (BDOI's text).</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Renewal FRS v1.1 final pass: every screen and walkthrough step recaptured on a fresh database, the channel connection address in business words, document prints at the standard width with wide extracts in two halves, no blank closing page, review checklist columns fitted; workbooks and coverage rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
@@ -4525,7 +4525,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Keep Clean / Review / Exception as the BRD says; show the Not for Renewal accounts as BDOI's "Non-Renewable" panel (a filter on the disposition). (BIBS reference FRS: FR-RN-022: buckets Clean, Review and Exception; missing mandatory data is a sanitation failure (Exception). The system today: Clean, Review, Exception.) Available in BIBS: the third panel of the renewal accounts is Non-Renewable (default, BDOI's panels Clean, Review, Non-Renewable and All, the Exception accounts shown under Review) or Exception (the BRD's Clean, Review and Exception).</t>
+          <t>Keep Clean / Review / Exception as the BRD says; show the Not for Renewal accounts as BDOI's "Non-Renewable" panel (a filter on the disposition). (The system today: Clean, Review, Exception.) Available in BIBS: the third panel of the renewal accounts is Non-Renewable (default, BDOI's panels Clean, Review, Non-Renewable and All, the Exception accounts shown under Review) or Exception (the BRD's Clean, Review and Exception).</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Keep the Review bucket (the TSU route is manual work) and use BDOI's disposition word once the For Quotation / For Proposal meaning is settled. (BIBS reference FRS: FR-RN-020: above PHP 250M the renewal account is Review and the decision matrix proposes For Proposal to TSU. The system today: Review with a proposed disposition.) Available in BIBS: an account above the sum insured threshold is Clean For Quotation and goes to the TSU (default, BDOI's rule) or Review with a proposal for the TSU.</t>
+          <t>Keep the Review bucket (the TSU route is manual work) and use BDOI's disposition word once the For Quotation / For Proposal meaning is settled. (The system today: Review with a proposed disposition.) Available in BIBS: an account above the sum insured threshold is Clean For Quotation and goes to the TSU (default, BDOI's rule) or Review with a proposal for the TSU.</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's meaning (BDOI's process vocabulary) after Marketing confirms it; the change to the system is the routing of the two values. (BIBS reference FRS: Dispositions table: For Quotation - a package quotation; For Proposal - a non-package proposal request (TSU). The system today: For Quotation to the package quotation, For Proposal to the proposal request.)</t>
+          <t>Adopt BDOI's meaning (BDOI's process vocabulary) after Marketing confirms it; the change to the system is the routing of the two values. (The system today: For Quotation to the package quotation, For Proposal to the proposal request.)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Ask BDOI which of its two rules applies; we recommend Annex C (renew in the open market) as the detailed rule, with the change of account type. (BIBS reference FRS: FR-RN-025: a paid-off loan tags the account Not for Renewal with reason "Loan fully paid". The system today: Not for Renewal, reason Loan fully paid.)</t>
+          <t>Ask BDOI which of its two rules applies; we recommend Annex C (renew in the open market) as the detailed rule, with the change of account type. (The system today: Not for Renewal, reason Loan fully paid.)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Ask BDOI; take RMU from the AO code list if LAMD sends the full loan list (FRRN.012). (BIBS reference FRS: FR-RN-025: RMU tags Not for Renewal with reason RMU, or transfers to the Corporate RMU unit; RMU comes from the LAMD report. The system today: Not for Renewal or transfer; RMU from the report.)</t>
+          <t>Ask BDOI; take RMU from the AO code list if LAMD sends the full loan list (FRRN.012). (The system today: Not for Renewal or transfer; RMU from the report.)</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Keep the Team Lead assignment of the BRD and add automatic assignment as an option per segment (change to the system), if BDOI confirms. (BIBS reference FRS: FR-RN-030, 061: the Team Lead assigns and re-assigns; CBG accounts are not assigned. The system today: Manual assignment.) Available in BIBS: the renewal accounts of the market segments chosen are assigned automatically to an Account Officer of the team, fewest open accounts first and then in turn, and the accounts routed to Processing to a Processing Officer when a second setting is on; with no segment chosen (default, the BRD) the Team Leader assigns.</t>
+          <t>Keep the Team Lead assignment of the BRD and add automatic assignment as an option per segment (change to the system), if BDOI confirms. (The system today: Manual assignment.) Available in BIBS: the renewal accounts of the market segments chosen are assigned automatically to an Account Officer of the team, fewest open accounts first and then in turn, and the accounts routed to Processing to a Processing Officer when a second setting is on; with no segment chosen (default, the BRD) the Team Leader assigns.</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD transfer; add BDOI's referral as a second action (New Business opportunity) if BDOI wants both. (BIBS reference FRS: FR-RN-031, 032: the renewal moves to the receiving unit when it accepts. The system today: Ownership transfer.) Available in BIBS: a transfer to another Marketing unit is a referral (the receiving unit opens a New Business account and the renewal keeps its owner, BDOI's text), a move of the account (the BRD), or both offered to the user (default).</t>
+          <t>Keep the BRD transfer; add BDOI's referral as a second action (New Business opportunity) if BDOI wants both. (The system today: Ownership transfer.) Available in BIBS: a transfer to another Marketing unit is a referral (the receiving unit opens a New Business account and the renewal keeps its owner, BDOI's text), a move of the account (the BRD), or both offered to the user (default).</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Keep both triggers; BDOI confirms the lead days per segment. (BIBS reference FRS: FR-RN-010, 011: a daily run extracts at 140 lead days (configurable); users also generate any range. The system today: Daily run and on-demand range.)</t>
+          <t>Keep both triggers; BDOI confirms the lead days per segment. (The system today: Daily run and on-demand range.)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Keep ours; use BDOI's status names on the renewal record (In Process Renewal for an initiated renewal). (BIBS reference FRS: FR-RN-010, 015, 063: extraction creates a renewal record; nothing starts until initiation; the renewal account is created when processing starts. The system today: Renewal record first, account at processing.)</t>
+          <t>Keep ours; use BDOI's status names on the renewal record (In Process Renewal for an initiated renewal). (The system today: Renewal record first, account at processing.)</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's nine values as a list mapped to the three BRD outcomes, with BDOI's bucket and disposition per value (change to the system). (BIBS reference FRS: FR-RN-071: Renew As Is, Revise, Reject; Reject tags Not for Renewal (insurer declined) or returns to Marketing. The system today: Three responses.)</t>
+          <t>Adopt BDOI's nine values as a list mapped to the three BRD outcomes, with BDOI's bucket and disposition per value (change to the system). (The system today: Three responses.)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Keep the RA lock of the BRD and add BDOI's lock after placement (edits after placement are already refused by the account). (BIBS reference FRS: FR-RN-080: RA generation locks the account on the Marketing side; an RA cancellation unlocks it. The system today: Lock at RA generation.) Available in BIBS: Marketing can no longer change the account once the Renewal Advice is generated (default, BDOI's text) or once it is posted and the placement is sent.</t>
+          <t>Keep the RA lock of the BRD and add BDOI's lock after placement (edits after placement are already refused by the account). (The system today: Lock at RA generation.) Available in BIBS: Marketing can no longer change the account once the Renewal Advice is generated (default, BDOI's text) or once it is posted and the placement is sent.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's durations as parameters now; automatic requests and extensions are a change to the system for BDOI to prioritise. (BIBS reference FRS: FR-RN-086: the user requests 30 or 60 days (default 30) when the renewal will not complete in time. The system today: User request, 30 or 60 days.) Available in BIBS: hold cover durations of 30 days (Non-CBG), 90 days (CBG), 60 days (CBG Motor after an insurer's rejection) and 30 days (CBG Home), extensions of 15 or 30 days from 7 days before the end, automatic requests for Non-CBG accounts after the client's confirmation and for Clean CBG accounts 75 days before expiry, and the monthly CBG Home extension on the 15th; each value is a setting.</t>
+          <t>Adopt BDOI's durations as parameters now; automatic requests and extensions are a change to the system for BDOI to prioritise. (The system today: User request, 30 or 60 days.) Available in BIBS: hold cover durations of 30 days (Non-CBG), 90 days (CBG), 60 days (CBG Motor after an insurer's rejection) and 30 days (CBG Home), extensions of 15 or 30 days from 7 days before the end, automatic requests for Non-CBG accounts after the client's confirmation and for Clean CBG accounts 75 days before expiry, and the monthly CBG Home extension on the 15th; each value is a setting.</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's 75 / 45 days and the automatic determination; name the notices First and Final as in the approved templates. (BIBS reference FRS: FR-RN-080: the user chooses First or Second Notice; second notice after 15 days without acceptance; warning below 30 days. The system today: User choice; second-notice days parameter.) Available in BIBS: the Renewal Advice notice follows the expiry, First Notice from 75 days and Last Notice from 45 days before expiry (default, BDOI's text), or is chosen by the user.</t>
+          <t>Adopt BDOI's 75 / 45 days and the automatic determination; name the notices First and Final as in the approved templates. (The system today: User choice; second-notice days parameter.) Available in BIBS: the Renewal Advice notice follows the expiry, First Notice from 75 days and Last Notice from 45 days before expiry (default, BDOI's text), or is chosen by the user.</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's definition and 75 days (parameter value). (BIBS reference FRS: FR-RN-083: accounts not yet submitted at the checkpoint, 90 days before expiry by default, all segments. The system today: 90-day parameter.)</t>
+          <t>Adopt BDOI's definition and 75 days (parameter value). (The system today: 90-day parameter.)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Keep the mutual exclusion and the effective expiry date of the BRD; adopt BDOI's day offsets (1 and 3 days) as parameters. (BIBS reference FRS: FR-RN-082: at the effective expiry date (hold cover end), NAL when an RA was sent, NRL when none; the two exclude each other. The system today: Mutually exclusive, effective expiry date.) Available in BIBS: the No Advice Letter 1 day and the Non-Renewal Letter 1 day (CBG Motor) or 3 days (Non-CBG) after the effective expiry date, each a setting; the two letters exclude each other.</t>
+          <t>Keep the mutual exclusion and the effective expiry date of the BRD; adopt BDOI's day offsets (1 and 3 days) as parameters. (The system today: Mutually exclusive, effective expiry date.) Available in BIBS: the No Advice Letter 1 day and the Non-Renewal Letter 1 day (CBG Motor) or 3 days (Non-CBG) after the effective expiry date, each a setting; the two letters exclude each other.</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's convention (answers Q07); change to the system of the password rule. (BIBS reference FRS: FR-RN-081: password convention per Q07; until then a generated password per e-mail. The system today: Random 12-character password in a separate e-mail.) Available in BIBS: protected files use BDOI's password convention (default: the first three letters of the first and last names in capitals for an individual client, eight random characters for a corporate client) or a random password per file.</t>
+          <t>Adopt BDOI's convention (answers Q07); change to the system of the password rule. (The system today: Random 12-character password in a separate e-mail.) Available in BIBS: protected files use BDOI's password convention (default: the first three letters of the first and last names in capitals for an individual client, eight random characters for a corporate client) or a random password per file.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>BDO ITG decides whether CCM and MFT are in scope for go-live; the system keeps e-mail as the fallback channel. (BIBS reference FRS: Outgoing e-mail, protected, with a send log; no file-transfer channel with insurers (on hold). The system today: Outgoing e-mail; CCM listed as an option in the integration inventory (IQ11).) Available in BIBS: client documents are sent through CCM (default) or by protected e-mail with the password in a separate e-mail; insurers receive their files through MFT when enrolled, otherwise by e-mail.</t>
+          <t>BDO ITG decides whether CCM and MFT are in scope for go-live; the system keeps e-mail as the fallback channel. (The system today: Outgoing e-mail; CCM listed as an option in the integration inventory (IQ11).) Available in BIBS: client documents are sent through CCM (default) or by protected e-mail with the password in a separate e-mail; insurers receive their files through MFT when enrolled, otherwise by e-mail.</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Keep ours; align BDOI's wording with BRRN.041. (BIBS reference FRS: FR-RN-087: after booking, confirmed acceptance and full payment. The system today: After booking and full payment.)</t>
+          <t>Keep ours; align BDOI's wording with BRRN.041. (The system today: After booking and full payment.)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Ask BDOI which timing it means; both are parameter values. (BIBS reference FRS: FR-RN-001: warning 30 minutes before the system-triggered log-out. The system today: Idle warning and log-out timings by parameter.)</t>
+          <t>Ask BDOI which timing it means; both are parameter values. (The system today: Idle warning and log-out timings by parameter.)</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Keep the booking a user action as the Walkthrough addendum says, unless BDOI changes it. (BIBS reference FRS: FR-RN-084: placement and booking stay user actions. The system today: Booking is a user action (automatic booking rules exist in New Business).) Available in BIBS: the insurer's approval of the placement leaves the account For Booking for the Processing Officer (default, the BRD) or books and locks it (BDOI's text).</t>
+          <t>Keep the booking a user action as the Walkthrough addendum says, unless BDOI changes it. (The system today: Booking is a user action (automatic booking rules exist in New Business).) Available in BIBS: the insurer's approval of the placement leaves the account For Booking for the Processing Officer (default, the BRD) or books and locks it (BDOI's text).</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Keep ours and add BDOI's Review routing for endorsements of the term if Marketing wants to see them. (BIBS reference FRS: FR-RN-027: posted endorsements are taken into the renewal; an endorsement in progress blocks post, RA and acceptance. The system today: Pending endorsement blocks.) Available in BIBS: every endorsement of the expiring term routes the account to Review (default, BDOI's text) or only an endorsement in progress.</t>
+          <t>Keep ours and add BDOI's Review routing for endorsements of the term if Marketing wants to see them. (The system today: Pending endorsement blocks.) Available in BIBS: every endorsement of the expiring term routes the account to Review (default, BDOI's text) or only an endorsement in progress.</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Keep the five dispositions of the BRD and add BDOI's eleven extra reasons as list values. (BIBS reference FRS: FR-RN-043: five dispositions (with Lost Business) and ten reasons. The system today: Five dispositions; eleven reasons (list values).) Available in BIBS: the dispositions offered to Marketing are For Renewal, Not for Renewal, For Quotation, For Proposal and Lost Business (default, the BRD) or the first four with Lost Business as a reason of Not for Renewal (BDOI's text); BDOI's non-renewal reasons are in the list of values.</t>
+          <t>Keep the five dispositions of the BRD and add BDOI's eleven extra reasons as list values. (The system today: Five dispositions; eleven reasons (list values).) Available in BIBS: the dispositions offered to Marketing are For Renewal, Not for Renewal, For Quotation, For Proposal and Lost Business (default, the BRD) or the first four with Lost Business as a reason of Not for Renewal (BDOI's text); BDOI's non-renewal reasons are in the list of values.</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Ask BDOI; a second approval is a change to the system and slows BRRN.040. (BIBS reference FRS: FR-RN-084: the accepted account moves to placement and booking without resubmission. The system today: No second approval.) Available in BIBS: an accepted account goes to the payment check and placement at once (default, the BRD) or is Submitted for Approval and goes to placement once an approver approves it (BDOI's text).</t>
+          <t>Ask BDOI; a second approval is a change to the system and slows BRRN.040. (The system today: No second approval.) Available in BIBS: an accepted account goes to the payment check and placement at once (default, the BRD) or is Submitted for Approval and goes to placement once an approver approves it (BDOI's text).</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Keep the matrix and load BDOI's rule (Clean is automatic For Renewal) as its first content. (BIBS reference FRS: FR-RN-023: the decision matrix gives a system disposition to Clean accounts whose rule is automatic; others are proposed to the AO; the Team Lead posts. The system today: Matrix proposal or automatic disposition.) Available in BIBS: Clean accounts are disposed For Renewal automatically (default, BDOI's rule) or wait for the disposition of Marketing.</t>
+          <t>Keep the matrix and load BDOI's rule (Clean is automatic For Renewal) as its first content. (The system today: Matrix proposal or automatic disposition.) Available in BIBS: Clean accounts are disposed For Renewal automatically (default, BDOI's rule) or wait for the disposition of Marketing.</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Map the two lists one to one in the status model annex and use BDOI's names where the BRD is silent. (BIBS reference FRS: Extracted, Evaluating, Unassigned Disposition, For Disposition, Review in Progress, For Processing, With Insurer, RA Ready, RA Sent, Accepted, For Placement and Booking, Renewed, Closed. The system today: The the system stages.) Available in BIBS: the statuses read with BDOI's names (default: In Process Renewal, Submitted for Posting, Posted and the others) or with the workflow status names.</t>
+          <t>Map the two lists one to one in the status model annex and use BDOI's names where the BRD is silent. (The system today: The the system stages.) Available in BIBS: the statuses read with BDOI's names (default: In Process Renewal, Submitted for Posting, Posted and the others) or with the workflow status names.</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Use BDOI's names RMEL and NRL in the merged FRS and on the screens. (BIBS reference FRS: Expiry List; Not for Renewal Letter (NFR). The system today: Expiry List; NAL / NFR.) Available in BIBS: generated files are named with BDOI's convention &lt;Product&gt;_&lt;Letter&gt;_&lt;Reference&gt;_MMDDYYYY.pdf (default) or with the letter number.</t>
+          <t>Use BDOI's names RMEL and NRL in the merged FRS and on the screens. (The system today: Expiry List; NAL / NFR.) Available in BIBS: generated files are named with BDOI's convention &lt;Product&gt;_&lt;Letter&gt;_&lt;Reference&gt;_MMDDYYYY.pdf (default) or with the letter number.</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD label and correct BDOI's two variants. (BIBS reference FRS: FR-RN-024: "Non-renewable Accounts". The system today: Non-renewable Accounts.) Available in BIBS: the reason recorded for a non-renewable risk code is Non-renewable Accounts (default, the BRD) or Non-Renewable Risk Code (BDOI's text).</t>
+          <t>Keep the BRD label and correct BDOI's two variants. (The system today: Non-renewable Accounts.) Available in BIBS: the reason recorded for a non-renewable risk code is Non-renewable Accounts (default, the BRD) or Non-Renewable Risk Code (BDOI's text).</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's automatic status change; the placement itself stays a user action. (BIBS reference FRS: FR-RN-084: the accepted renewal moves to placement and booking when the payment rules are met; automatic placement is off for renewals. The system today: Fast track to placement; placement by the user.)</t>
+          <t>Adopt BDOI's automatic status change; the placement itself stays a user action. (The system today: Fast track to placement; placement by the user.)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Renewal FRS v1.2: colour code of the points beyond the BRD (green out of the box, orange change request) with its legend, Annex AP.1 with the CR effort, CR Effort Estimate workbook, register and RTM scope columns, Concept Paper traced (Annex AM.4), programme NFRs of other BRDs in Annex AJ, environment of screenshots and walkthroughs, figures kept with captions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to use'!$A$4:$D$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to use'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$U$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
@@ -796,7 +796,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>BRD-06 Renewal - after the sign-off of the FRS v1.1</t>
+          <t>BRD-06 Renewal - after the sign-off of the FRS v1.2</t>
         </is>
       </c>
     </row>
@@ -939,11 +939,11 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Candidate changes known at v1.1 (status Candidate - for decision) and new requests</t>
+          <t>Candidate changes known at v1.2: green (out of the box, no cost) and orange (effort in the CR Effort Estimate workbook)</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1384,15 +1384,15 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr"/>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Raised, Candidate - for decision, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
-        </is>
-      </c>
+          <t>FRS colour</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Green: beyond the BRD, out of the box (no cost); Orange: change request with effort</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
@@ -1402,15 +1402,15 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>Decision of the approvers</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr"/>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Raised, Candidate - for decision, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -1420,10 +1420,14 @@
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>Approved by</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Decision of the approvers</t>
+        </is>
+      </c>
       <c r="D25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1434,7 +1438,7 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>Decision date</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr"/>
@@ -1448,7 +1452,7 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Target drop</t>
+          <t>Decision date</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr"/>
@@ -1462,30 +1466,26 @@
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>Linked test cases</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Test cases of the Test Cases and Traceability workbook</t>
-        </is>
-      </c>
+          <t>Target drop</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr"/>
       <c r="D28" s="14" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Impact assessment form</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Linked test cases</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Part of the assessment</t>
+          <t>Test cases of the Test Cases and Traceability workbook</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr"/>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>Assessment</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Filled in by the project</t>
+          <t>Part of the assessment</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr"/>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>Assessed by</t>
+          <t>Assessment</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Filled in by the project</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr"/>
@@ -1529,17 +1529,17 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Decisions log</t>
+          <t>Impact assessment form</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>Annex AO No.</t>
+          <t>Assessed by</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Row of Annex AO of the FRS v1.1</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr"/>
@@ -1552,10 +1552,14 @@
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr"/>
+          <t>Annex AO No.</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Row of Annex AO of the FRS v1.2</t>
+        </is>
+      </c>
       <c r="D33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1566,7 +1570,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>Topic</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr"/>
@@ -1580,7 +1584,7 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Proposed in the FRS</t>
+          <t>Topic</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr"/>
@@ -1594,7 +1598,7 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>Decision by</t>
+          <t>Proposed in the FRS</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr"/>
@@ -1608,14 +1612,10 @@
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>Adopt proposal / Keep BDOI text / Other</t>
-        </is>
-      </c>
+          <t>Decision by</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr"/>
       <c r="D37" s="12" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1626,10 +1626,14 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>Decided by (name)</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Adopt proposal / Keep BDOI text / Other</t>
+        </is>
+      </c>
       <c r="D38" s="14" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1640,7 +1644,7 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Decided by (name)</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr"/>
@@ -1654,7 +1658,7 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>CR No. (if a change follows)</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr"/>
@@ -1668,18 +1672,32 @@
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
+          <t>CR No. (if a change follows)</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr"/>
+      <c r="D41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Decisions log</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr"/>
-      <c r="D41" s="12" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr"/>
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>Open, Decided, Withdrawn</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D41"/>
+  <autoFilter ref="A4:D42"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -1913,7 +1931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1930,12 +1948,13 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1948,7 +1967,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Candidate changes known at v1.1 (status Candidate - for decision) and new requests</t>
+          <t>Candidate changes known at v1.2: green (out of the box, no cost) and orange (effort in the CR Effort Estimate workbook)</t>
         </is>
       </c>
     </row>
@@ -1973,6 +1992,7 @@
       <c r="R3" s="23" t="n"/>
       <c r="S3" s="23" t="n"/>
       <c r="T3" s="23" t="n"/>
+      <c r="U3" s="23" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2047,30 +2067,35 @@
       </c>
       <c r="O4" s="24" t="inlineStr">
         <is>
+          <t>FRS colour</t>
+        </is>
+      </c>
+      <c r="P4" s="24" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="P4" s="24" t="inlineStr">
+      <c r="Q4" s="24" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="Q4" s="24" t="inlineStr">
+      <c r="R4" s="24" t="inlineStr">
         <is>
           <t>Approved by</t>
         </is>
       </c>
-      <c r="R4" s="24" t="inlineStr">
+      <c r="S4" s="24" t="inlineStr">
         <is>
           <t>Decision date</t>
         </is>
       </c>
-      <c r="S4" s="24" t="inlineStr">
+      <c r="T4" s="24" t="inlineStr">
         <is>
           <t>Target drop</t>
         </is>
       </c>
-      <c r="T4" s="24" t="inlineStr">
+      <c r="U4" s="24" t="inlineStr">
         <is>
           <t>Linked test cases</t>
         </is>
@@ -2124,12 +2149,12 @@
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K5" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
@@ -2147,16 +2172,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="O5" s="25" t="inlineStr">
+      <c r="O5" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-01)</t>
+        </is>
+      </c>
+      <c r="P5" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P5" s="12" t="inlineStr"/>
       <c r="Q5" s="12" t="inlineStr"/>
       <c r="R5" s="12" t="inlineStr"/>
       <c r="S5" s="12" t="inlineStr"/>
-      <c r="T5" s="12" t="inlineStr">
+      <c r="T5" s="12" t="inlineStr"/>
+      <c r="U5" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-010-01-AC01, TC-FRRN-010-01-AC02, TC-FRRN-010-01-AC03, TC-RN-030.1-01, TC-RN-030.1-02</t>
         </is>
@@ -2210,39 +2240,44 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.011 cases</t>
+        </is>
+      </c>
+      <c r="N6" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L6" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M6" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.011 cases</t>
-        </is>
-      </c>
-      <c r="N6" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
+      <c r="O6" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-02)</t>
+        </is>
+      </c>
+      <c r="P6" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P6" s="12" t="inlineStr"/>
       <c r="Q6" s="12" t="inlineStr"/>
       <c r="R6" s="12" t="inlineStr"/>
       <c r="S6" s="12" t="inlineStr"/>
-      <c r="T6" s="12" t="inlineStr">
+      <c r="T6" s="12" t="inlineStr"/>
+      <c r="U6" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-011-03-AC01</t>
         </is>
@@ -2296,12 +2331,12 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
@@ -2319,16 +2354,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O7" s="25" t="inlineStr">
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-03)</t>
+        </is>
+      </c>
+      <c r="P7" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P7" s="12" t="inlineStr"/>
       <c r="Q7" s="12" t="inlineStr"/>
       <c r="R7" s="12" t="inlineStr"/>
       <c r="S7" s="12" t="inlineStr"/>
-      <c r="T7" s="12" t="inlineStr">
+      <c r="T7" s="12" t="inlineStr"/>
+      <c r="U7" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-002-02-01-AC01, TC-FRRN-002-02-01-AC02</t>
         </is>
@@ -2382,39 +2422,44 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.003.02 cases</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M8" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.003.02 cases</t>
-        </is>
-      </c>
-      <c r="N8" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O8" s="25" t="inlineStr">
+      <c r="O8" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-04)</t>
+        </is>
+      </c>
+      <c r="P8" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P8" s="12" t="inlineStr"/>
       <c r="Q8" s="12" t="inlineStr"/>
       <c r="R8" s="12" t="inlineStr"/>
       <c r="S8" s="12" t="inlineStr"/>
-      <c r="T8" s="12" t="inlineStr">
+      <c r="T8" s="12" t="inlineStr"/>
+      <c r="U8" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-003-02-AC01, TC-FRRN-003-02-AC02</t>
         </is>
@@ -2468,39 +2513,44 @@
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.042 cases</t>
+        </is>
+      </c>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.042 cases</t>
-        </is>
-      </c>
-      <c r="N9" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O9" s="25" t="inlineStr">
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-05)</t>
+        </is>
+      </c>
+      <c r="P9" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P9" s="12" t="inlineStr"/>
       <c r="Q9" s="12" t="inlineStr"/>
       <c r="R9" s="12" t="inlineStr"/>
       <c r="S9" s="12" t="inlineStr"/>
-      <c r="T9" s="12" t="inlineStr">
+      <c r="T9" s="12" t="inlineStr"/>
+      <c r="U9" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-042-01-AC01</t>
         </is>
@@ -2554,39 +2604,44 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>Customer Servicing</t>
+        </is>
+      </c>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.039 cases</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
-        <is>
-          <t>Customer Servicing</t>
-        </is>
-      </c>
-      <c r="M10" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.039 cases</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O10" s="25" t="inlineStr">
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-06)</t>
+        </is>
+      </c>
+      <c r="P10" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P10" s="12" t="inlineStr"/>
       <c r="Q10" s="12" t="inlineStr"/>
       <c r="R10" s="12" t="inlineStr"/>
       <c r="S10" s="12" t="inlineStr"/>
-      <c r="T10" s="12" t="inlineStr">
+      <c r="T10" s="12" t="inlineStr"/>
+      <c r="U10" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-039-02-AC01</t>
         </is>
@@ -2640,12 +2695,12 @@
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
@@ -2663,16 +2718,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O11" s="25" t="inlineStr">
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-07)</t>
+        </is>
+      </c>
+      <c r="P11" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P11" s="12" t="inlineStr"/>
       <c r="Q11" s="12" t="inlineStr"/>
       <c r="R11" s="12" t="inlineStr"/>
       <c r="S11" s="12" t="inlineStr"/>
-      <c r="T11" s="12" t="inlineStr">
+      <c r="T11" s="12" t="inlineStr"/>
+      <c r="U11" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-012-06-AC01, TC-FRRN-012-06-AC02</t>
         </is>
@@ -2726,39 +2786,44 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>Product Maintenance</t>
+        </is>
+      </c>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.009.01 cases</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K12" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L12" s="12" t="inlineStr">
-        <is>
-          <t>Product Maintenance</t>
-        </is>
-      </c>
-      <c r="M12" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.009.01 cases</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O12" s="25" t="inlineStr">
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-08)</t>
+        </is>
+      </c>
+      <c r="P12" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P12" s="12" t="inlineStr"/>
       <c r="Q12" s="12" t="inlineStr"/>
       <c r="R12" s="12" t="inlineStr"/>
       <c r="S12" s="12" t="inlineStr"/>
-      <c r="T12" s="12" t="inlineStr">
+      <c r="T12" s="12" t="inlineStr"/>
+      <c r="U12" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-009-01-AC01, TC-FRRN-009-01-AC02, TC-FRRN-009-01-AC03, TC-RN-063.1-01, TC-RN-063.2-01</t>
         </is>
@@ -2812,39 +2877,44 @@
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M13" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.014.03 cases</t>
+        </is>
+      </c>
+      <c r="N13" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M13" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.014.03 cases</t>
-        </is>
-      </c>
-      <c r="N13" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O13" s="25" t="inlineStr">
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-09)</t>
+        </is>
+      </c>
+      <c r="P13" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P13" s="12" t="inlineStr"/>
       <c r="Q13" s="12" t="inlineStr"/>
       <c r="R13" s="12" t="inlineStr"/>
       <c r="S13" s="12" t="inlineStr"/>
-      <c r="T13" s="12" t="inlineStr">
+      <c r="T13" s="12" t="inlineStr"/>
+      <c r="U13" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-014-03-AC01, TC-FRRN-014-03-AC02</t>
         </is>
@@ -2898,12 +2968,12 @@
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L14" s="12" t="inlineStr">
@@ -2921,16 +2991,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O14" s="25" t="inlineStr">
+      <c r="O14" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-10)</t>
+        </is>
+      </c>
+      <c r="P14" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P14" s="12" t="inlineStr"/>
       <c r="Q14" s="12" t="inlineStr"/>
       <c r="R14" s="12" t="inlineStr"/>
       <c r="S14" s="12" t="inlineStr"/>
-      <c r="T14" s="12" t="inlineStr">
+      <c r="T14" s="12" t="inlineStr"/>
+      <c r="U14" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-014-05-AC01, TC-FRRN-014-05-AC02</t>
         </is>
@@ -2984,39 +3059,44 @@
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.036 cases</t>
+        </is>
+      </c>
+      <c r="N15" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K15" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M15" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.036 cases</t>
-        </is>
-      </c>
-      <c r="N15" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O15" s="25" t="inlineStr">
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-11)</t>
+        </is>
+      </c>
+      <c r="P15" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P15" s="12" t="inlineStr"/>
       <c r="Q15" s="12" t="inlineStr"/>
       <c r="R15" s="12" t="inlineStr"/>
       <c r="S15" s="12" t="inlineStr"/>
-      <c r="T15" s="12" t="inlineStr">
+      <c r="T15" s="12" t="inlineStr"/>
+      <c r="U15" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-036-03-AC01</t>
         </is>
@@ -3070,39 +3150,44 @@
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>All BRDs that send e-mail</t>
+        </is>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>Sending cases</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>All BRDs that send e-mail</t>
-        </is>
-      </c>
-      <c r="M16" s="12" t="inlineStr">
-        <is>
-          <t>Sending cases</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O16" s="25" t="inlineStr">
+      <c r="O16" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-12)</t>
+        </is>
+      </c>
+      <c r="P16" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P16" s="12" t="inlineStr"/>
       <c r="Q16" s="12" t="inlineStr"/>
       <c r="R16" s="12" t="inlineStr"/>
       <c r="S16" s="12" t="inlineStr"/>
-      <c r="T16" s="12" t="inlineStr">
+      <c r="T16" s="12" t="inlineStr"/>
+      <c r="U16" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-022-02-AC01, TC-FRRN-022-02-AC02, TC-RN-081.1-01, TC-RN-081.1-02, TC-RN-081.1-03</t>
         </is>
@@ -3156,12 +3241,12 @@
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
@@ -3179,16 +3264,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O17" s="25" t="inlineStr">
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-13)</t>
+        </is>
+      </c>
+      <c r="P17" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P17" s="12" t="inlineStr"/>
       <c r="Q17" s="12" t="inlineStr"/>
       <c r="R17" s="12" t="inlineStr"/>
       <c r="S17" s="12" t="inlineStr"/>
-      <c r="T17" s="12" t="inlineStr">
+      <c r="T17" s="12" t="inlineStr"/>
+      <c r="U17" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-29-03-AC01</t>
         </is>
@@ -3242,39 +3332,44 @@
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M18" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.033 cases</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K18" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L18" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M18" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.033 cases</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O18" s="25" t="inlineStr">
+      <c r="O18" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-14)</t>
+        </is>
+      </c>
+      <c r="P18" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P18" s="12" t="inlineStr"/>
       <c r="Q18" s="12" t="inlineStr"/>
       <c r="R18" s="12" t="inlineStr"/>
       <c r="S18" s="12" t="inlineStr"/>
-      <c r="T18" s="12" t="inlineStr">
+      <c r="T18" s="12" t="inlineStr"/>
+      <c r="U18" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-033-01-AC01</t>
         </is>
@@ -3328,12 +3423,12 @@
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -3351,16 +3446,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O19" s="25" t="inlineStr">
+      <c r="O19" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-15)</t>
+        </is>
+      </c>
+      <c r="P19" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P19" s="12" t="inlineStr"/>
       <c r="Q19" s="12" t="inlineStr"/>
       <c r="R19" s="12" t="inlineStr"/>
       <c r="S19" s="12" t="inlineStr"/>
-      <c r="T19" s="12" t="inlineStr">
+      <c r="T19" s="12" t="inlineStr"/>
+      <c r="U19" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-29-05-AC01, TC-FRRN-29-05-AC02, TC-RN-070.1-01, TC-RN-070.1-02, TC-RN-070.2-01</t>
         </is>
@@ -3414,12 +3514,12 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L20" s="12" t="inlineStr">
@@ -3437,16 +3537,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="O20" s="25" t="inlineStr">
+      <c r="O20" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-16)</t>
+        </is>
+      </c>
+      <c r="P20" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P20" s="12" t="inlineStr"/>
       <c r="Q20" s="12" t="inlineStr"/>
       <c r="R20" s="12" t="inlineStr"/>
       <c r="S20" s="12" t="inlineStr"/>
-      <c r="T20" s="12" t="inlineStr">
+      <c r="T20" s="12" t="inlineStr"/>
+      <c r="U20" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-26-01-AC01, TC-FRRN-26-01-AC02</t>
         </is>
@@ -3500,12 +3605,12 @@
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
@@ -3523,16 +3628,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="O21" s="25" t="inlineStr">
+      <c r="O21" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-17)</t>
+        </is>
+      </c>
+      <c r="P21" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P21" s="12" t="inlineStr"/>
       <c r="Q21" s="12" t="inlineStr"/>
       <c r="R21" s="12" t="inlineStr"/>
       <c r="S21" s="12" t="inlineStr"/>
-      <c r="T21" s="12" t="inlineStr">
+      <c r="T21" s="12" t="inlineStr"/>
+      <c r="U21" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-013-02-AC01, TC-FRRN-013-02-AC02, TC-FRRN-013-02-AC03, TC-RN-071.1-01, TC-RN-071.2-01</t>
         </is>
@@ -3586,39 +3696,44 @@
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>New Business</t>
+        </is>
+      </c>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.006.01 cases</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K22" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L22" s="12" t="inlineStr">
-        <is>
-          <t>New Business</t>
-        </is>
-      </c>
-      <c r="M22" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.006.01 cases</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O22" s="25" t="inlineStr">
+      <c r="O22" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-18)</t>
+        </is>
+      </c>
+      <c r="P22" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P22" s="12" t="inlineStr"/>
       <c r="Q22" s="12" t="inlineStr"/>
       <c r="R22" s="12" t="inlineStr"/>
       <c r="S22" s="12" t="inlineStr"/>
-      <c r="T22" s="12" t="inlineStr">
+      <c r="T22" s="12" t="inlineStr"/>
+      <c r="U22" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-006-01-AC01, TC-FRRN-006-01-AC02, TC-FRRN-006-01-AC03</t>
         </is>
@@ -3672,12 +3787,12 @@
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
@@ -3695,16 +3810,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="O23" s="25" t="inlineStr">
+      <c r="O23" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-19)</t>
+        </is>
+      </c>
+      <c r="P23" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P23" s="12" t="inlineStr"/>
       <c r="Q23" s="12" t="inlineStr"/>
       <c r="R23" s="12" t="inlineStr"/>
       <c r="S23" s="12" t="inlineStr"/>
-      <c r="T23" s="12" t="inlineStr">
+      <c r="T23" s="12" t="inlineStr"/>
+      <c r="U23" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-022-01-AC01, TC-FRRN-022-01-AC02, TC-FRRN-022-01-AC03, TC-FRRN-022-01-AC04, TC-RN-080.1-01</t>
         </is>
@@ -3758,12 +3878,12 @@
       </c>
       <c r="J24" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -3781,16 +3901,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="O24" s="25" t="inlineStr">
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-20)</t>
+        </is>
+      </c>
+      <c r="P24" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P24" s="12" t="inlineStr"/>
       <c r="Q24" s="12" t="inlineStr"/>
       <c r="R24" s="12" t="inlineStr"/>
       <c r="S24" s="12" t="inlineStr"/>
-      <c r="T24" s="12" t="inlineStr">
+      <c r="T24" s="12" t="inlineStr"/>
+      <c r="U24" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-024-01-AC01, TC-FRRN-024-01-AC02, TC-FRRN-024-01-AC03, TC-RN-081.1-01, TC-RN-081.1-02</t>
         </is>
@@ -3844,39 +3969,44 @@
       </c>
       <c r="J25" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>New Business; Cashiering</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.027 cases</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K25" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>New Business; Cashiering</t>
-        </is>
-      </c>
-      <c r="M25" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.027 cases</t>
-        </is>
-      </c>
-      <c r="N25" s="12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="O25" s="25" t="inlineStr">
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-21)</t>
+        </is>
+      </c>
+      <c r="P25" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P25" s="12" t="inlineStr"/>
       <c r="Q25" s="12" t="inlineStr"/>
       <c r="R25" s="12" t="inlineStr"/>
       <c r="S25" s="12" t="inlineStr"/>
-      <c r="T25" s="12" t="inlineStr">
+      <c r="T25" s="12" t="inlineStr"/>
+      <c r="U25" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-27-01-AC01, TC-FRRN-27-01-AC02</t>
         </is>
@@ -3930,12 +4060,12 @@
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>To assess</t>
+          <t>None - out of the box</t>
         </is>
       </c>
       <c r="L26" s="12" t="inlineStr">
@@ -3953,16 +4083,21 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O26" s="25" t="inlineStr">
+      <c r="O26" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-22)</t>
+        </is>
+      </c>
+      <c r="P26" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P26" s="12" t="inlineStr"/>
       <c r="Q26" s="12" t="inlineStr"/>
       <c r="R26" s="12" t="inlineStr"/>
       <c r="S26" s="12" t="inlineStr"/>
-      <c r="T26" s="12" t="inlineStr">
+      <c r="T26" s="12" t="inlineStr"/>
+      <c r="U26" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-041-01-AC01, TC-FRRN-041-01-AC02, TC-RN-025.1-01, TC-RN-025.2-01, TC-RN-025.2-02</t>
         </is>
@@ -4016,67 +4151,163 @@
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>None - out of the box</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>User Access Maintenance</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>FRRN.043 cases</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr">
-        <is>
-          <t>To assess</t>
-        </is>
-      </c>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>User Access Maintenance</t>
-        </is>
-      </c>
-      <c r="M27" s="12" t="inlineStr">
-        <is>
-          <t>FRRN.043 cases</t>
-        </is>
-      </c>
-      <c r="N27" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O27" s="25" t="inlineStr">
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>Green (G-23)</t>
+        </is>
+      </c>
+      <c r="P27" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="P27" s="12" t="inlineStr"/>
       <c r="Q27" s="12" t="inlineStr"/>
       <c r="R27" s="12" t="inlineStr"/>
       <c r="S27" s="12" t="inlineStr"/>
-      <c r="T27" s="12" t="inlineStr">
+      <c r="T27" s="12" t="inlineStr"/>
+      <c r="U27" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-043-01-AC01, TC-FRRN-043-01-AC02, TC-RN-004.1-01, TC-RN-004.2-01, TC-RN-004.3-01</t>
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>CR-RN-024</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>Annex AJ RN-NFR-16</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Accessibility conformance (WCAG 2.2 level AA) of the Renewal screens</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>The BRD has no accessibility requirement; BDO's policies and the programme register expect screens usable with the keyboard and a screen reader, with sufficient contrast. A conformance claim needs a check of every Renewal screen and the corrections it finds.</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Renewal screens</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>To plan</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>20.0 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>Shared screen components</t>
+        </is>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>New accessibility checks</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="P28" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="Q28" s="12" t="inlineStr"/>
+      <c r="R28" s="12" t="inlineStr"/>
+      <c r="S28" s="12" t="inlineStr"/>
+      <c r="T28" s="12" t="inlineStr"/>
+      <c r="U28" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:T27"/>
+  <autoFilter ref="A4:U28"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A2:U2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:O527">
+  <conditionalFormatting sqref="P5:P528">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:T527">
+  <conditionalFormatting sqref="A5:U528">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H5:H527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="H5:H528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="N5:N528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="P5:P528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Renewal FRS v1.2 on rules v2: out of the box tested against the iNXT BrokerVerse platform edition (3 green, 17 orange CRs of 153.0 man-days, 4 integration-scope points with grey labels), best-practice annex AP.2 in blue, legend with black/green/orange/grey/blue; effort workbook sheets Summary, CR Effort, Beyond the BRD - OOTB, Integration & DM scope, Best practice, BRD items to deliver, Assumptions (DayRate); register and RTM aligned; Fit-Gap column names iNXT BrokerVerse
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to use'!$A$4:$D$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to use'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$U$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$V$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1384,12 +1384,12 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>FRS colour</t>
+          <t>Feature List ID / OOTB status</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Green: beyond the BRD, out of the box (no cost); Orange: change request with effort</t>
+          <t>Feature List vs OOTB, column OOTB platform</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr"/>
@@ -1402,15 +1402,15 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Raised, Candidate - for decision, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
-        </is>
-      </c>
+          <t>FRS colour</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Green: beyond the BRD, out of the box (no cost); Orange: change request with effort; Grey: Integration or Data Migration scope</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -1420,15 +1420,15 @@
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>Decision of the approvers</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr"/>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr"/>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Raised, Candidate - for decision, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -1438,10 +1438,14 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>Approved by</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Decision of the approvers</t>
+        </is>
+      </c>
       <c r="D26" s="14" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1452,7 +1456,7 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Decision date</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr"/>
@@ -1466,7 +1470,7 @@
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>Target drop</t>
+          <t>Decision date</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr"/>
@@ -1480,30 +1484,26 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Linked test cases</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>Test cases of the Test Cases and Traceability workbook</t>
-        </is>
-      </c>
+          <t>Target drop</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr"/>
       <c r="D29" s="12" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Impact assessment form</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Linked test cases</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Part of the assessment</t>
+          <t>Test cases of the Test Cases and Traceability workbook</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr"/>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>Assessment</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Filled in by the project</t>
+          <t>Part of the assessment</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>Assessed by</t>
+          <t>Assessment</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Filled in by the project</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr"/>
@@ -1547,17 +1547,17 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Decisions log</t>
+          <t>Impact assessment form</t>
         </is>
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Annex AO No.</t>
+          <t>Assessed by</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Row of Annex AO of the FRS v1.2</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr"/>
@@ -1570,10 +1570,14 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr"/>
+          <t>Annex AO No.</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Row of Annex AO of the FRS v1.2</t>
+        </is>
+      </c>
       <c r="D34" s="14" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1584,7 +1588,7 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Topic</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr"/>
@@ -1598,7 +1602,7 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>Proposed in the FRS</t>
+          <t>Topic</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr"/>
@@ -1612,7 +1616,7 @@
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Decision by</t>
+          <t>Proposed in the FRS</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr"/>
@@ -1626,14 +1630,10 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>Adopt proposal / Keep BDOI text / Other</t>
-        </is>
-      </c>
+          <t>Decision by</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr"/>
       <c r="D38" s="14" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1644,10 +1644,14 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Decided by (name)</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Adopt proposal / Keep BDOI text / Other</t>
+        </is>
+      </c>
       <c r="D39" s="12" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1658,7 +1662,7 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Decided by (name)</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr"/>
@@ -1672,7 +1676,7 @@
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>CR No. (if a change follows)</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr"/>
@@ -1686,18 +1690,32 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
+          <t>CR No. (if a change follows)</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr"/>
+      <c r="D42" s="14" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Decisions log</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr"/>
-      <c r="D42" s="14" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr"/>
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>Open, Decided, Withdrawn</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D42"/>
+  <autoFilter ref="A4:D43"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -1931,7 +1949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1948,13 +1966,14 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1993,6 +2012,7 @@
       <c r="S3" s="23" t="n"/>
       <c r="T3" s="23" t="n"/>
       <c r="U3" s="23" t="n"/>
+      <c r="V3" s="23" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2067,35 +2087,40 @@
       </c>
       <c r="O4" s="24" t="inlineStr">
         <is>
+          <t>Feature List ID / OOTB status</t>
+        </is>
+      </c>
+      <c r="P4" s="24" t="inlineStr">
+        <is>
           <t>FRS colour</t>
         </is>
       </c>
-      <c r="P4" s="24" t="inlineStr">
+      <c r="Q4" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="Q4" s="24" t="inlineStr">
+      <c r="R4" s="24" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="R4" s="24" t="inlineStr">
+      <c r="S4" s="24" t="inlineStr">
         <is>
           <t>Approved by</t>
         </is>
       </c>
-      <c r="S4" s="24" t="inlineStr">
+      <c r="T4" s="24" t="inlineStr">
         <is>
           <t>Decision date</t>
         </is>
       </c>
-      <c r="T4" s="24" t="inlineStr">
+      <c r="U4" s="24" t="inlineStr">
         <is>
           <t>Target drop</t>
         </is>
       </c>
-      <c r="U4" s="24" t="inlineStr">
+      <c r="V4" s="24" t="inlineStr">
         <is>
           <t>Linked test cases</t>
         </is>
@@ -2149,12 +2174,12 @@
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K5" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>6.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
@@ -2174,19 +2199,24 @@
       </c>
       <c r="O5" s="12" t="inlineStr">
         <is>
-          <t>Green (G-01)</t>
-        </is>
-      </c>
-      <c r="P5" s="25" t="inlineStr">
+          <t>RNW-012: Partial</t>
+        </is>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q5" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr"/>
       <c r="R5" s="12" t="inlineStr"/>
       <c r="S5" s="12" t="inlineStr"/>
       <c r="T5" s="12" t="inlineStr"/>
-      <c r="U5" s="12" t="inlineStr">
+      <c r="U5" s="12" t="inlineStr"/>
+      <c r="V5" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-010-01-AC01, TC-FRRN-010-01-AC02, TC-FRRN-010-01-AC03, TC-RN-030.1-01, TC-RN-030.1-02</t>
         </is>
@@ -2240,12 +2270,12 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>10.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L6" s="12" t="inlineStr">
@@ -2265,19 +2295,24 @@
       </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>Green (G-02)</t>
-        </is>
-      </c>
-      <c r="P6" s="25" t="inlineStr">
+          <t>RNW-013: Not available</t>
+        </is>
+      </c>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q6" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr"/>
       <c r="R6" s="12" t="inlineStr"/>
       <c r="S6" s="12" t="inlineStr"/>
       <c r="T6" s="12" t="inlineStr"/>
-      <c r="U6" s="12" t="inlineStr">
+      <c r="U6" s="12" t="inlineStr"/>
+      <c r="V6" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-011-03-AC01</t>
         </is>
@@ -2331,12 +2366,12 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>9.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
@@ -2356,19 +2391,24 @@
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>Green (G-03)</t>
-        </is>
-      </c>
-      <c r="P7" s="25" t="inlineStr">
+          <t>RNW-032; ACC-023: Partial</t>
+        </is>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q7" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr"/>
       <c r="R7" s="12" t="inlineStr"/>
       <c r="S7" s="12" t="inlineStr"/>
       <c r="T7" s="12" t="inlineStr"/>
-      <c r="U7" s="12" t="inlineStr">
+      <c r="U7" s="12" t="inlineStr"/>
+      <c r="V7" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-002-02-01-AC01, TC-FRRN-002-02-01-AC02</t>
         </is>
@@ -2422,12 +2462,12 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>9.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L8" s="12" t="inlineStr">
@@ -2447,19 +2487,24 @@
       </c>
       <c r="O8" s="12" t="inlineStr">
         <is>
-          <t>Green (G-04)</t>
-        </is>
-      </c>
-      <c r="P8" s="25" t="inlineStr">
+          <t>QPL-032: Partial</t>
+        </is>
+      </c>
+      <c r="P8" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q8" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr"/>
       <c r="R8" s="12" t="inlineStr"/>
       <c r="S8" s="12" t="inlineStr"/>
       <c r="T8" s="12" t="inlineStr"/>
-      <c r="U8" s="12" t="inlineStr">
+      <c r="U8" s="12" t="inlineStr"/>
+      <c r="V8" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-003-02-AC01, TC-FRRN-003-02-AC02</t>
         </is>
@@ -2513,12 +2558,12 @@
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>11.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L9" s="12" t="inlineStr">
@@ -2538,19 +2583,24 @@
       </c>
       <c r="O9" s="12" t="inlineStr">
         <is>
-          <t>Green (G-05)</t>
-        </is>
-      </c>
-      <c r="P9" s="25" t="inlineStr">
+          <t>ACC-023: Not available</t>
+        </is>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q9" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr"/>
       <c r="R9" s="12" t="inlineStr"/>
       <c r="S9" s="12" t="inlineStr"/>
       <c r="T9" s="12" t="inlineStr"/>
-      <c r="U9" s="12" t="inlineStr">
+      <c r="U9" s="12" t="inlineStr"/>
+      <c r="V9" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-042-01-AC01</t>
         </is>
@@ -2604,12 +2654,12 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>8.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -2624,24 +2674,29 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Green (G-06)</t>
-        </is>
-      </c>
-      <c r="P10" s="25" t="inlineStr">
+          <t>RNW-010; CRM-010: Partial</t>
+        </is>
+      </c>
+      <c r="P10" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q10" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr"/>
       <c r="R10" s="12" t="inlineStr"/>
       <c r="S10" s="12" t="inlineStr"/>
       <c r="T10" s="12" t="inlineStr"/>
-      <c r="U10" s="12" t="inlineStr">
+      <c r="U10" s="12" t="inlineStr"/>
+      <c r="V10" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-039-02-AC01</t>
         </is>
@@ -2685,22 +2740,22 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>BDOFC and BDOSOLD reports of BDO systems</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Integration plan</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>Not a CR - Integration scope</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
@@ -2720,19 +2775,24 @@
       </c>
       <c r="O11" s="12" t="inlineStr">
         <is>
-          <t>Green (G-07)</t>
-        </is>
-      </c>
-      <c r="P11" s="25" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" s="12" t="inlineStr">
+        <is>
+          <t>Grey label (Integration scope)</t>
+        </is>
+      </c>
+      <c r="Q11" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr"/>
       <c r="R11" s="12" t="inlineStr"/>
       <c r="S11" s="12" t="inlineStr"/>
       <c r="T11" s="12" t="inlineStr"/>
-      <c r="U11" s="12" t="inlineStr">
+      <c r="U11" s="12" t="inlineStr"/>
+      <c r="V11" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-012-06-AC01, TC-FRRN-012-06-AC02</t>
         </is>
@@ -2786,12 +2846,12 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>11.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L12" s="12" t="inlineStr">
@@ -2811,19 +2871,24 @@
       </c>
       <c r="O12" s="12" t="inlineStr">
         <is>
-          <t>Green (G-08)</t>
-        </is>
-      </c>
-      <c r="P12" s="25" t="inlineStr">
+          <t>Not in the feature list: BDOI-specific</t>
+        </is>
+      </c>
+      <c r="P12" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q12" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr"/>
       <c r="R12" s="12" t="inlineStr"/>
       <c r="S12" s="12" t="inlineStr"/>
       <c r="T12" s="12" t="inlineStr"/>
-      <c r="U12" s="12" t="inlineStr">
+      <c r="U12" s="12" t="inlineStr"/>
+      <c r="V12" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-009-01-AC01, TC-FRRN-009-01-AC02, TC-FRRN-009-01-AC03, TC-RN-063.1-01, TC-RN-063.2-01</t>
         </is>
@@ -2902,19 +2967,24 @@
       </c>
       <c r="O13" s="12" t="inlineStr">
         <is>
+          <t>QPL-016: Available</t>
+        </is>
+      </c>
+      <c r="P13" s="12" t="inlineStr">
+        <is>
           <t>Green (G-09)</t>
         </is>
       </c>
-      <c r="P13" s="25" t="inlineStr">
+      <c r="Q13" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr"/>
       <c r="R13" s="12" t="inlineStr"/>
       <c r="S13" s="12" t="inlineStr"/>
       <c r="T13" s="12" t="inlineStr"/>
-      <c r="U13" s="12" t="inlineStr">
+      <c r="U13" s="12" t="inlineStr"/>
+      <c r="V13" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-014-03-AC01, TC-FRRN-014-03-AC02</t>
         </is>
@@ -2968,12 +3038,12 @@
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>6.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L14" s="12" t="inlineStr">
@@ -2993,19 +3063,24 @@
       </c>
       <c r="O14" s="12" t="inlineStr">
         <is>
-          <t>Green (G-10)</t>
-        </is>
-      </c>
-      <c r="P14" s="25" t="inlineStr">
+          <t>POL-016; REM-019: Partial</t>
+        </is>
+      </c>
+      <c r="P14" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q14" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr"/>
       <c r="R14" s="12" t="inlineStr"/>
       <c r="S14" s="12" t="inlineStr"/>
       <c r="T14" s="12" t="inlineStr"/>
-      <c r="U14" s="12" t="inlineStr">
+      <c r="U14" s="12" t="inlineStr"/>
+      <c r="V14" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-014-05-AC01, TC-FRRN-014-05-AC02</t>
         </is>
@@ -3059,12 +3134,12 @@
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>15.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
@@ -3079,24 +3154,29 @@
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>Green (G-11)</t>
-        </is>
-      </c>
-      <c r="P15" s="25" t="inlineStr">
+          <t>RNW-028: Partial</t>
+        </is>
+      </c>
+      <c r="P15" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q15" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr"/>
       <c r="R15" s="12" t="inlineStr"/>
       <c r="S15" s="12" t="inlineStr"/>
       <c r="T15" s="12" t="inlineStr"/>
-      <c r="U15" s="12" t="inlineStr">
+      <c r="U15" s="12" t="inlineStr"/>
+      <c r="V15" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-036-03-AC01</t>
         </is>
@@ -3145,17 +3225,17 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Sending</t>
+          <t>CCM of BDO (client communications)</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Integration plan</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>Not a CR - Integration scope</t>
         </is>
       </c>
       <c r="L16" s="12" t="inlineStr">
@@ -3175,19 +3255,24 @@
       </c>
       <c r="O16" s="12" t="inlineStr">
         <is>
-          <t>Green (G-12)</t>
-        </is>
-      </c>
-      <c r="P16" s="25" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" s="12" t="inlineStr">
+        <is>
+          <t>Grey label (Integration scope)</t>
+        </is>
+      </c>
+      <c r="Q16" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr"/>
       <c r="R16" s="12" t="inlineStr"/>
       <c r="S16" s="12" t="inlineStr"/>
       <c r="T16" s="12" t="inlineStr"/>
-      <c r="U16" s="12" t="inlineStr">
+      <c r="U16" s="12" t="inlineStr"/>
+      <c r="V16" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-022-02-AC01, TC-FRRN-022-02-AC02, TC-RN-081.1-01, TC-RN-081.1-02, TC-RN-081.1-03</t>
         </is>
@@ -3236,17 +3321,17 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Insurer exchange</t>
+          <t>MFT with the insurers</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Integration plan</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>Not a CR - Integration scope</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
@@ -3266,19 +3351,24 @@
       </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>Green (G-13)</t>
-        </is>
-      </c>
-      <c r="P17" s="25" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" s="12" t="inlineStr">
+        <is>
+          <t>Grey label (Integration scope)</t>
+        </is>
+      </c>
+      <c r="Q17" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr"/>
       <c r="R17" s="12" t="inlineStr"/>
       <c r="S17" s="12" t="inlineStr"/>
       <c r="T17" s="12" t="inlineStr"/>
-      <c r="U17" s="12" t="inlineStr">
+      <c r="U17" s="12" t="inlineStr"/>
+      <c r="V17" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-29-03-AC01</t>
         </is>
@@ -3332,12 +3422,12 @@
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>10.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L18" s="12" t="inlineStr">
@@ -3357,19 +3447,24 @@
       </c>
       <c r="O18" s="12" t="inlineStr">
         <is>
-          <t>Green (G-14)</t>
-        </is>
-      </c>
-      <c r="P18" s="25" t="inlineStr">
+          <t>POL-009: Partial</t>
+        </is>
+      </c>
+      <c r="P18" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q18" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr"/>
       <c r="R18" s="12" t="inlineStr"/>
       <c r="S18" s="12" t="inlineStr"/>
       <c r="T18" s="12" t="inlineStr"/>
-      <c r="U18" s="12" t="inlineStr">
+      <c r="U18" s="12" t="inlineStr"/>
+      <c r="V18" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-033-01-AC01</t>
         </is>
@@ -3423,12 +3518,12 @@
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>8.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -3448,19 +3543,24 @@
       </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>Green (G-15)</t>
-        </is>
-      </c>
-      <c r="P19" s="25" t="inlineStr">
+          <t>QPL-032 (no TAT feature): Not available</t>
+        </is>
+      </c>
+      <c r="P19" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q19" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr"/>
       <c r="R19" s="12" t="inlineStr"/>
       <c r="S19" s="12" t="inlineStr"/>
       <c r="T19" s="12" t="inlineStr"/>
-      <c r="U19" s="12" t="inlineStr">
+      <c r="U19" s="12" t="inlineStr"/>
+      <c r="V19" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-29-05-AC01, TC-FRRN-29-05-AC02, TC-RN-070.1-01, TC-RN-070.1-02, TC-RN-070.2-01</t>
         </is>
@@ -3514,12 +3614,12 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>6.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L20" s="12" t="inlineStr">
@@ -3534,24 +3634,29 @@
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr">
         <is>
-          <t>Green (G-16)</t>
-        </is>
-      </c>
-      <c r="P20" s="25" t="inlineStr">
+          <t>RNW-016: Partial</t>
+        </is>
+      </c>
+      <c r="P20" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q20" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr"/>
       <c r="R20" s="12" t="inlineStr"/>
       <c r="S20" s="12" t="inlineStr"/>
       <c r="T20" s="12" t="inlineStr"/>
-      <c r="U20" s="12" t="inlineStr">
+      <c r="U20" s="12" t="inlineStr"/>
+      <c r="V20" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-26-01-AC01, TC-FRRN-26-01-AC02</t>
         </is>
@@ -3605,12 +3710,12 @@
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>6.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
@@ -3625,24 +3730,29 @@
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>Green (G-17)</t>
-        </is>
-      </c>
-      <c r="P21" s="25" t="inlineStr">
+          <t>RNW-021: BDOI-specific</t>
+        </is>
+      </c>
+      <c r="P21" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q21" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr"/>
       <c r="R21" s="12" t="inlineStr"/>
       <c r="S21" s="12" t="inlineStr"/>
       <c r="T21" s="12" t="inlineStr"/>
-      <c r="U21" s="12" t="inlineStr">
+      <c r="U21" s="12" t="inlineStr"/>
+      <c r="V21" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-013-02-AC01, TC-FRRN-013-02-AC02, TC-FRRN-013-02-AC03, TC-RN-071.1-01, TC-RN-071.2-01</t>
         </is>
@@ -3696,12 +3806,12 @@
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>5.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L22" s="12" t="inlineStr">
@@ -3721,19 +3831,24 @@
       </c>
       <c r="O22" s="12" t="inlineStr">
         <is>
-          <t>Green (G-18)</t>
-        </is>
-      </c>
-      <c r="P22" s="25" t="inlineStr">
+          <t>POL-003: Partial</t>
+        </is>
+      </c>
+      <c r="P22" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q22" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr"/>
       <c r="R22" s="12" t="inlineStr"/>
       <c r="S22" s="12" t="inlineStr"/>
       <c r="T22" s="12" t="inlineStr"/>
-      <c r="U22" s="12" t="inlineStr">
+      <c r="U22" s="12" t="inlineStr"/>
+      <c r="V22" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-006-01-AC01, TC-FRRN-006-01-AC02, TC-FRRN-006-01-AC03</t>
         </is>
@@ -3812,19 +3927,24 @@
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
+          <t>RNW-022: Available</t>
+        </is>
+      </c>
+      <c r="P23" s="12" t="inlineStr">
+        <is>
           <t>Green (G-19)</t>
         </is>
       </c>
-      <c r="P23" s="25" t="inlineStr">
+      <c r="Q23" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr"/>
       <c r="R23" s="12" t="inlineStr"/>
       <c r="S23" s="12" t="inlineStr"/>
       <c r="T23" s="12" t="inlineStr"/>
-      <c r="U23" s="12" t="inlineStr">
+      <c r="U23" s="12" t="inlineStr"/>
+      <c r="V23" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-022-01-AC01, TC-FRRN-022-01-AC02, TC-FRRN-022-01-AC03, TC-FRRN-022-01-AC04, TC-RN-080.1-01</t>
         </is>
@@ -3878,12 +3998,12 @@
       </c>
       <c r="J24" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>4.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -3903,19 +4023,24 @@
       </c>
       <c r="O24" s="12" t="inlineStr">
         <is>
-          <t>Green (G-20)</t>
-        </is>
-      </c>
-      <c r="P24" s="25" t="inlineStr">
+          <t>RNW-023; QPL-031: Not available</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q24" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr"/>
       <c r="R24" s="12" t="inlineStr"/>
       <c r="S24" s="12" t="inlineStr"/>
       <c r="T24" s="12" t="inlineStr"/>
-      <c r="U24" s="12" t="inlineStr">
+      <c r="U24" s="12" t="inlineStr"/>
+      <c r="V24" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-024-01-AC01, TC-FRRN-024-01-AC02, TC-FRRN-024-01-AC03, TC-RN-081.1-01, TC-RN-081.1-02</t>
         </is>
@@ -3964,17 +4089,17 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>CLPC billing files to BDO CBG Loan Services (LMS)</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Integration plan</t>
         </is>
       </c>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>Not a CR - Integration scope</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr">
@@ -3994,19 +4119,24 @@
       </c>
       <c r="O25" s="12" t="inlineStr">
         <is>
-          <t>Green (G-21)</t>
-        </is>
-      </c>
-      <c r="P25" s="25" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr">
+        <is>
+          <t>Grey label (Integration scope)</t>
+        </is>
+      </c>
+      <c r="Q25" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr"/>
       <c r="R25" s="12" t="inlineStr"/>
       <c r="S25" s="12" t="inlineStr"/>
       <c r="T25" s="12" t="inlineStr"/>
-      <c r="U25" s="12" t="inlineStr">
+      <c r="U25" s="12" t="inlineStr"/>
+      <c r="V25" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-27-01-AC01, TC-FRRN-27-01-AC02</t>
         </is>
@@ -4060,12 +4190,12 @@
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>To plan</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>None - out of the box</t>
+          <t>5.0 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L26" s="12" t="inlineStr">
@@ -4080,24 +4210,29 @@
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O26" s="12" t="inlineStr">
         <is>
-          <t>Green (G-22)</t>
-        </is>
-      </c>
-      <c r="P26" s="25" t="inlineStr">
+          <t>RNW-009; INT-009: BDOI-specific</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="Q26" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q26" s="12" t="inlineStr"/>
       <c r="R26" s="12" t="inlineStr"/>
       <c r="S26" s="12" t="inlineStr"/>
       <c r="T26" s="12" t="inlineStr"/>
-      <c r="U26" s="12" t="inlineStr">
+      <c r="U26" s="12" t="inlineStr"/>
+      <c r="V26" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-041-01-AC01, TC-FRRN-041-01-AC02, TC-RN-025.1-01, TC-RN-025.2-01, TC-RN-025.2-02</t>
         </is>
@@ -4176,19 +4311,24 @@
       </c>
       <c r="O27" s="12" t="inlineStr">
         <is>
+          <t>RNW-037: Available</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr">
+        <is>
           <t>Green (G-23)</t>
         </is>
       </c>
-      <c r="P27" s="25" t="inlineStr">
+      <c r="Q27" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q27" s="12" t="inlineStr"/>
       <c r="R27" s="12" t="inlineStr"/>
       <c r="S27" s="12" t="inlineStr"/>
       <c r="T27" s="12" t="inlineStr"/>
-      <c r="U27" s="12" t="inlineStr">
+      <c r="U27" s="12" t="inlineStr"/>
+      <c r="V27" s="12" t="inlineStr">
         <is>
           <t>TC-FRRN-043-01-AC01, TC-FRRN-043-01-AC02, TC-RN-004.1-01, TC-RN-004.2-01, TC-RN-004.3-01</t>
         </is>
@@ -4267,35 +4407,40 @@
       </c>
       <c r="O28" s="12" t="inlineStr">
         <is>
+          <t>NFR-021: Partial</t>
+        </is>
+      </c>
+      <c r="P28" s="12" t="inlineStr">
+        <is>
           <t>Orange</t>
         </is>
       </c>
-      <c r="P28" s="25" t="inlineStr">
+      <c r="Q28" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q28" s="12" t="inlineStr"/>
       <c r="R28" s="12" t="inlineStr"/>
       <c r="S28" s="12" t="inlineStr"/>
       <c r="T28" s="12" t="inlineStr"/>
-      <c r="U28" s="12" t="inlineStr">
+      <c r="U28" s="12" t="inlineStr"/>
+      <c r="V28" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:U28"/>
+  <autoFilter ref="A4:V28"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A2:V2"/>
   </mergeCells>
-  <conditionalFormatting sqref="P5:P528">
+  <conditionalFormatting sqref="Q5:Q528">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:U528">
+  <conditionalFormatting sqref="A5:V528">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
@@ -4307,7 +4452,7 @@
     <dataValidation sqref="N5:N528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="P5:P528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="Q5:Q528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Orange only for points in no BRD: Renewal v1.2 and User Access Maintenance v1.4 re-classified against the BRD lines
Renewal: 13 former CRs are BRD requirements (black, BRD items to deliver, 102.5 man-days) and CR-RN-008 split
(field update 5.0 to deliver; Annexes D/E rules 6.5 stay orange); 4 orange CRs of 45.5 man-days.
User Access Maintenance: CR-UA-008, 009, 013 are BRD (BRD-UA-18 to 20); CR-UA-011 and 014 split (BRD-UA-21, 22);
5 orange CRs of 53.0 man-days; end-to-end flow tags, register, RTM and effort workbooks rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-06_Renewal/BIBS_CR_BRD-06_Change_Request_Register_v1.0.xlsx
@@ -2144,7 +2144,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>BRD 1.005, 3.005</t>
+          <t>BRD 1.005.1, 3.005; BRRN.031</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS; the BRD has the Team Lead's assignment</t>
+          <t>In the BRD: BRD 1.005.1 "a. Assign account to Marketing Account Officers (AO)"; BRD 3.005 (assignment to the Processing Officer); BRRN.031 "apply rule-based disposition automatically ... so that straight-through renewals proceed without manual effort"</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -2169,17 +2169,17 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Assignment rules and the hierarchy of Annex F</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K5" s="12" t="inlineStr">
         <is>
-          <t>6.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (6.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
@@ -2204,17 +2204,25 @@
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R5" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R5" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S5" s="12" t="inlineStr"/>
-      <c r="T5" s="12" t="inlineStr"/>
+      <c r="T5" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U5" s="12" t="inlineStr"/>
       <c r="V5" s="12" t="inlineStr">
         <is>
@@ -2240,7 +2248,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>BRD 1.006</t>
+          <t>BRD 1.006, 1.007.3; BRRN.033</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -2255,7 +2263,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS; the BRD transfers the account</t>
+          <t>In the BRD: BRD 1.006 "Transfer account to other units" (1.006.3 "Select from the drop-down the Marketing unit where the account will be transferred to", 1.006.4 "Submit transfer request"); BRD 1.007.3 "Accept transferred account/s"; BRRN.033 "allow renewal-identified accounts to follow the New Business flow"</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -2265,17 +2273,17 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>Transfer and New Business</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>10.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (10.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L6" s="12" t="inlineStr">
@@ -2300,17 +2308,25 @@
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q6" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R6" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S6" s="12" t="inlineStr"/>
-      <c r="T6" s="12" t="inlineStr"/>
+      <c r="T6" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U6" s="12" t="inlineStr"/>
       <c r="V6" s="12" t="inlineStr">
         <is>
@@ -2336,7 +2352,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>BRD 1.009.7</t>
+          <t>BRD 1.009.7; BRRN.021; BRD-00 BR-203</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2351,7 +2367,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS beyond BRD 1.009.7</t>
+          <t>In the BRD: BRD 1.009.7 "g. View the assigned accounts per Marketing AO in a dashboard"; BRRN.021 "displayed on the screen/dashboard"; BRD-00 BR-203 "Dashboards and reports for real-time tracking and reporting"</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -2361,17 +2377,17 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>9.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (9.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
@@ -2396,17 +2412,25 @@
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q7" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R7" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S7" s="12" t="inlineStr"/>
-      <c r="T7" s="12" t="inlineStr"/>
+      <c r="T7" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U7" s="12" t="inlineStr"/>
       <c r="V7" s="12" t="inlineStr">
         <is>
@@ -2432,7 +2456,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>BRD 3.010.7</t>
+          <t>BRD 3.010.7; BRD-00 BR-203</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -2447,7 +2471,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS beyond BRD 3.010.7</t>
+          <t>In the BRD: BRD 3.010.7 "g. View the assigned accounts per Processing Officer in a dashboard"; BRD-00 BR-203 "Dashboards and reports for real-time tracking and reporting"</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
@@ -2457,17 +2481,17 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>9.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (9.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L8" s="12" t="inlineStr">
@@ -2492,17 +2516,25 @@
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q8" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R8" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S8" s="12" t="inlineStr"/>
-      <c r="T8" s="12" t="inlineStr"/>
+      <c r="T8" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U8" s="12" t="inlineStr"/>
       <c r="V8" s="12" t="inlineStr">
         <is>
@@ -2639,7 +2671,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS beyond the KYC flag</t>
+          <t>In the BRD: BRRN.028 "I want the system to identify and view accounts that are due or upcoming for KYC review, so that compliance monitoring and follow up can be performed without blocking or interrupting the renewal process"</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -2649,17 +2681,17 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>KYC</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>8.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (8.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -2674,7 +2706,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr">
@@ -2684,17 +2716,25 @@
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q10" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R10" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S10" s="12" t="inlineStr"/>
-      <c r="T10" s="12" t="inlineStr"/>
+      <c r="T10" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U10" s="12" t="inlineStr"/>
       <c r="V10" s="12" t="inlineStr">
         <is>
@@ -2826,7 +2866,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>CBG Motor automatic update: Depreciation, BI / PD tiers, Auto Promo to Regular (Annexes D, E)</t>
+          <t>CBG Motor automatic update: CBG Motor rules of Annexes D and E only: depreciation schedule of the sum insured, BI / PD tier table and the Auto Promo to Regular conversion</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -2851,7 +2891,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>11.5 man-days (CR Effort Estimate)</t>
+          <t>6.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
       <c r="L12" s="12" t="inlineStr">
@@ -3008,7 +3048,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>BRRN.040</t>
+          <t>BRD 2.004.4.4; BRD-00 BR-035</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -3023,7 +3063,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS</t>
+          <t>In the BRD: BRD 2.004.4.4 "4. Direct to Insurer" (reason for non-renewal); BRD-00 BR-035 "allow user to tag of Direct Payment (DP)"</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -3033,17 +3073,17 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>Approvals</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>6.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (6.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L14" s="12" t="inlineStr">
@@ -3068,17 +3108,25 @@
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q14" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R14" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S14" s="12" t="inlineStr"/>
-      <c r="T14" s="12" t="inlineStr"/>
+      <c r="T14" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U14" s="12" t="inlineStr"/>
       <c r="V14" s="12" t="inlineStr">
         <is>
@@ -3104,7 +3152,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>BRRN.042</t>
+          <t>BRRN.042; BRD-00 BR-034</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -3119,7 +3167,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS beyond BRRN.042</t>
+          <t>In the BRD: BRRN.042 "I want to be able to send request for Hold Cover to insurer/s and to record the Hold Cover confirmation details received from the insurer"; BRD-00 BR-034 "the system sends a 30 days Hold Cover (HC) request to Insurer/s"</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -3129,17 +3177,17 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Hold cover</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>15.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (15.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
@@ -3154,7 +3202,7 @@
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O15" s="12" t="inlineStr">
@@ -3164,17 +3212,25 @@
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q15" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R15" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R15" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S15" s="12" t="inlineStr"/>
-      <c r="T15" s="12" t="inlineStr"/>
+      <c r="T15" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U15" s="12" t="inlineStr"/>
       <c r="V15" s="12" t="inlineStr">
         <is>
@@ -3392,7 +3448,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>BRRN.040</t>
+          <t>BRD-00 BR-040 to BR-042; BRRN.040</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -3407,7 +3463,7 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS</t>
+          <t>In the BRD: BRD-00 BR-040 "allow users to receive e-policy. (Individual or Batch)", BR-041 "send e-policy to client. (Individual or Batch)", BR-042 "updates client record to add e-policy and policy number. (Individual or Batch)"; BRRN.040 "the policy can be issued on time"</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
@@ -3417,17 +3473,17 @@
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>Issuance</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>10.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (10.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L18" s="12" t="inlineStr">
@@ -3452,17 +3508,25 @@
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q18" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R18" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R18" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S18" s="12" t="inlineStr"/>
-      <c r="T18" s="12" t="inlineStr"/>
+      <c r="T18" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U18" s="12" t="inlineStr"/>
       <c r="V18" s="12" t="inlineStr">
         <is>
@@ -3584,7 +3648,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>BRRN.040</t>
+          <t>BRD 1.008.1, 1.009.3.2.10; BRRN.038</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -3599,7 +3663,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS; BRRN.040 asks for no delay</t>
+          <t>In the BRD: BRD 1.008.1 "Review and Post Disposition Accounts - a. Review Accounts"; BRD 1.009.3.2.10 "Total No. of Awaiting Marketing TL Approval (For Renewal)"; BRRN.038 "routing of renewal changes based on financial impact, ensuring proper approval"</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -3609,17 +3673,17 @@
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>6.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (6.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L20" s="12" t="inlineStr">
@@ -3634,7 +3698,7 @@
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr">
@@ -3644,17 +3708,25 @@
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q20" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R20" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R20" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S20" s="12" t="inlineStr"/>
-      <c r="T20" s="12" t="inlineStr"/>
+      <c r="T20" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U20" s="12" t="inlineStr"/>
       <c r="V20" s="12" t="inlineStr">
         <is>
@@ -3695,7 +3767,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS; the BRD has three outcomes</t>
+          <t>In the BRD: BRRN.035 "capture insurer responses (e.g., Approve/ Renew As-Is, Reject, Revise) and automatically apply them to the renewal workflow"</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -3705,17 +3777,17 @@
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>Insurer responses</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>6.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (6.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
@@ -3730,7 +3802,7 @@
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O21" s="12" t="inlineStr">
@@ -3740,17 +3812,25 @@
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q21" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R21" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R21" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S21" s="12" t="inlineStr"/>
-      <c r="T21" s="12" t="inlineStr"/>
+      <c r="T21" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U21" s="12" t="inlineStr"/>
       <c r="V21" s="12" t="inlineStr">
         <is>
@@ -3776,7 +3856,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>BRRN.005</t>
+          <t>BRRN.005; BRD-00 BR-026</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -3791,7 +3871,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS</t>
+          <t>In the BRD: BRRN.005 negative scenario "List contains duplicate or irrelevant accounts"; BRD-00 BR-026 "sanitize ... based on configurable business rules ... such as duplicate detection"</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -3801,17 +3881,17 @@
       </c>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>Sanitation</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>5.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (5.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L22" s="12" t="inlineStr">
@@ -3836,17 +3916,25 @@
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q22" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R22" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R22" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S22" s="12" t="inlineStr"/>
-      <c r="T22" s="12" t="inlineStr"/>
+      <c r="T22" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U22" s="12" t="inlineStr"/>
       <c r="V22" s="12" t="inlineStr">
         <is>
@@ -3968,7 +4056,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>BRRN.010</t>
+          <t>BRRN.010; BRD 1.010.7.1</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -3983,7 +4071,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS</t>
+          <t>In the BRD: BRRN.010 "Send RA in batch, with encryption and password protection"; BRD 1.010.7.1 "1. Encrypt and add password prior to sending"</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -3993,17 +4081,17 @@
       </c>
       <c r="I24" s="12" t="inlineStr">
         <is>
-          <t>Protection of files</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J24" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>4.5 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (4.5 man-days, planning)</t>
         </is>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -4028,17 +4116,25 @@
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q24" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R24" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R24" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S24" s="12" t="inlineStr"/>
-      <c r="T24" s="12" t="inlineStr"/>
+      <c r="T24" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U24" s="12" t="inlineStr"/>
       <c r="V24" s="12" t="inlineStr">
         <is>
@@ -4160,7 +4256,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>BRRN.029</t>
+          <t>BRD 2.004.4.1; BRRN.029</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -4175,7 +4271,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS</t>
+          <t>In the BRD: BRD 2.004.4.1 "1. Remedial Management Unit (RMU)"; BRRN.029 "ingest LAMD-provided reports and match paid-off loan records ... to determine renewal eligibility and proper routing"</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -4185,17 +4281,17 @@
       </c>
       <c r="I26" s="12" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>In scope (BRD)</t>
         </is>
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>To plan</t>
+          <t>Delivery plan</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>5.0 man-days (CR Effort Estimate)</t>
+          <t>Not a CR - BRD item to deliver (5.0 man-days, planning)</t>
         </is>
       </c>
       <c r="L26" s="12" t="inlineStr">
@@ -4210,7 +4306,7 @@
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O26" s="12" t="inlineStr">
@@ -4220,17 +4316,25 @@
       </c>
       <c r="P26" s="12" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Black (in the BRD)</t>
         </is>
       </c>
       <c r="Q26" s="25" t="inlineStr">
         <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="R26" s="12" t="inlineStr"/>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="R26" s="12" t="inlineStr">
+        <is>
+          <t>Closed as a change request: BRD requirement, delivered in scope (sheet BRD items to deliver of the CR Effort Estimate)</t>
+        </is>
+      </c>
       <c r="S26" s="12" t="inlineStr"/>
-      <c r="T26" s="12" t="inlineStr"/>
+      <c r="T26" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
       <c r="U26" s="12" t="inlineStr"/>
       <c r="V26" s="12" t="inlineStr">
         <is>
@@ -7781,7 +7885,7 @@
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>Kept as BDOI's requirements; the New Business FRS specifies the shared placement, issuance and billing; the change request register lists them as candidates so that BDOI confirms their priority.</t>
+          <t>Kept as BDOI's requirements. The dashboard metrics elaborate BRD 1.009.7 and 3.010.7 and the e-policy batch elaborates BR-040 to BR-042 of the programme BRD: BRD items to deliver (Annex AP.1). The budget maintenance (FRRN.042) is in no BRD and stays a change request; the New Business FRS specifies the shared placement, issuance and billing.</t>
         </is>
       </c>
       <c r="E85" s="12" t="inlineStr">

</xml_diff>